<commit_message>
Consolidar todo el contenido del Excel en una sola hoja (casos COSAL + RGP + resumen cobertura)
Agent-Logs-Url: https://github.com/SusanaMManrique/Legal_Defensa/sessions/d00509ac-95e9-449c-b16b-d5a8ab3949df

Co-authored-by: SusanaMManrique <262415683+SusanaMManrique@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Plan_Pruebas_PAC.xlsx
+++ b/Plan_Pruebas_PAC.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan de Pruebas PAC" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen Cobertura" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Casos PAC" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +42,11 @@
     <font>
       <b val="1"/>
       <color rgb="00548235"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00404040"/>
       <sz val="12"/>
     </font>
     <font>
@@ -97,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -113,10 +117,11 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -484,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -887,227 +892,206 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>RESUMEN DE COBERTURA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Aspecto cubierto</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>COSAL</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>RGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Alta expediente</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Caso 1 (manual)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Caso 1 (desde RGP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Flujo completo confirmación</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Caso 1</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Caso 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Rechazo</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Caso 2 (Fase 06, CMYC)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Caso 2 (Fase 08, ALBA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Solicitud aclaraciones</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Caso 3 (Fase 03, ALBA)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Caso 3 (Fase 05, ALJA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>CRUD materiales/expediente</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Caso 4</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Caso 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Informes obligatorios + firma</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Casos 1, 3</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Casos 1, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Documentos + permisos</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Caso 1 (Fases 07, 10)</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Caso 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Correos electrónicos</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Caso 1 (Fases 01→02, 05→07, 06→07)</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Caso 1 (Fases 01→02, 05→07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Pruebas negativas (permisos)</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Caso 4</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Caso 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Mando orgánico (excepción)</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Casos 1 y 3</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Casos 1 y 3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A10:G10"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>RESUMEN DE COBERTURA</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Aspecto cubierto</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>COSAL</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>RGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Alta expediente</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Caso 1 (manual)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Caso 1 (desde RGP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Flujo completo confirmación</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Caso 1</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Caso 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Rechazo</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Caso 2 (Fase 06, CMYC)</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Caso 2 (Fase 08, ALBA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Solicitud aclaraciones</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Caso 3 (Fase 03, ALBA)</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Caso 3 (Fase 05, ALJA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>CRUD materiales/expediente</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Caso 4</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Caso 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Informes obligatorios + firma</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Casos 1, 3</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Casos 1, 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Documentos + permisos</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Caso 1 (Fases 07, 10)</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Caso 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Correos electrónicos</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Caso 1 (Fases 01→02, 05→07, 06→07)</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Caso 1 (Fases 01→02, 05→07)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Pruebas negativas (permisos)</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Caso 4</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Caso 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Mando orgánico (excepción)</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Casos 1 y 3</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Casos 1 y 3</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A18:G18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>